<commit_message>
Étape 4 : variations, service Commentaire, contrôle littéral, évaluations H1-ancrage et H2
- contexte ciblé en trois rubriques balisées, filtre temporel (BF6) dans la requête SQL
- client LLM local (Ollama 127.0.0.1 / llama-cpp), température 0, JSON avec une nouvelle tentative
- mode extractif (--llm none) déterministe et signalé ; abstention visible
- contrôle de citation littérale R0-R3 sur constats et perspectives, traçabilité des sources
- évaluations H1-ancrage, H2 (TFR, typologie, échantillon de relecture), choix du LLM :
  « non mesuré » sans modèle de langage ; analyse réelle des commentaires publiés
- tableaux : libellés sur deux lignes, unité des lignes de dénombrement
- tests : 20+ cas d'harmonisation, exclusions, variations, filtre temporel, JSON invalide, réseau

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JXMEQCNGgRjDzvz3X6fC9
</commit_message>
<xml_diff>
--- a/data/pairing/a_valider_2021.xlsx
+++ b/data/pairing/a_valider_2021.xlsx
@@ -720,10 +720,10 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Congo | 2018 = -4,8
-Congo | 2019 = -0,1
-Congo | 2020 = -7,9
-Congo | 2021(e) = -1,2
+          <t>République du Congo | 2018 = -4,8
+République du Congo | 2019 = -0,1
+République du Congo | 2020 = -7,9
+République du Congo | 2021(e) = -1,2
 Gabon | 2018 = 0,8
 Gabon | 2019 = 3,9
 Gabon | 2020 = -1,8

</xml_diff>